<commit_message>
fix: correct data import & add month filter functionality
- Fix seed.py column matching: use 3-letter month abbreviations + position
  fallback for mislabeled columns (Apr 2025 net was 'marnet' duplicate)
  → FAAC rows: 3180 → 4587, cumulative total now £37.85T
- Fix Nasarawa spelling in SQL import files
- Add fetchMonthlySummary() querying faac_allocations directly for month
  filtering (was UI-only, never reached DB)
- Add hasIgrData to KpiData, gate IGR ratio display
- All fetch functions now accept optional month param
</commit_message>
<xml_diff>
--- a/FAAC_Allocation_Aggregated_2016-2026.xlsx
+++ b/FAAC_Allocation_Aggregated_2016-2026.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\FAAC\Dashboard\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Downloads\FAAC\faac-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3720010A-8531-4340-82AA-90258D8EF42E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7521977E-EC40-43BB-8E1A-DF52B6463984}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2016" sheetId="8" r:id="rId1"/>
@@ -24,6 +24,7 @@
     <sheet name="2024" sheetId="13" r:id="rId9"/>
     <sheet name="2025" sheetId="14" r:id="rId10"/>
     <sheet name="2026" sheetId="15" r:id="rId11"/>
+    <sheet name="Sheet1" sheetId="16" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="190">
   <si>
     <t>S/N</t>
   </si>
@@ -605,7 +606,13 @@
     <t>Total IGR USD</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t>Total net for now</t>
+  </si>
+  <si>
+    <t>total faac</t>
+  </si>
+  <si>
+    <t>aprnet</t>
   </si>
 </sst>
 </file>
@@ -1228,8 +1235,9 @@
         <f>AA2/253</f>
         <v>120782008.9143676</v>
       </c>
-      <c r="AD2" s="13" t="s">
-        <v>187</v>
+      <c r="AD2" s="13">
+        <f>AB2/253</f>
+        <v>132274008.11859922</v>
       </c>
     </row>
     <row r="3" spans="1:30" ht="15" x14ac:dyDescent="0.35">
@@ -1320,7 +1328,7 @@
         <v>32545358238.423405</v>
       </c>
       <c r="AC3" s="11">
-        <f t="shared" ref="AC3:AC38" si="2">AA3/253</f>
+        <f t="shared" ref="AC3:AC39" si="2">AA3/253</f>
         <v>117470107.83653915</v>
       </c>
       <c r="AD3" s="13">
@@ -4645,6 +4653,16 @@
       <c r="AD38" s="13">
         <f t="shared" si="3"/>
         <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AA39" s="10">
+        <f>SUM(AA2:AA38)</f>
+        <v>1349974624338.7173</v>
+      </c>
+      <c r="AC39" s="11">
+        <f t="shared" si="2"/>
+        <v>5335868080.3901873</v>
       </c>
     </row>
     <row r="40" spans="1:30" x14ac:dyDescent="0.3">
@@ -4685,11 +4703,11 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE31D74A-5412-46B6-AB36-7C6066297840}">
-  <dimension ref="A1:AC38"/>
+  <dimension ref="A1:AC39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="26" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4722,7 +4740,7 @@
         <v>75</v>
       </c>
       <c r="J1" t="s">
-        <v>155</v>
+        <v>189</v>
       </c>
       <c r="K1" t="s">
         <v>77</v>
@@ -4954,7 +4972,7 @@
         <v>168340791845.63</v>
       </c>
       <c r="AB3" s="13">
-        <f t="shared" ref="AB3:AB38" si="1">AA3/1544</f>
+        <f t="shared" ref="AB3:AB39" si="1">AA3/1544</f>
         <v>109029010.26271373</v>
       </c>
     </row>
@@ -8012,6 +8030,16 @@
       <c r="AB38" s="13">
         <f t="shared" si="1"/>
         <v>132239724.14382124</v>
+      </c>
+    </row>
+    <row r="39" spans="1:28" x14ac:dyDescent="0.3">
+      <c r="AA39" s="13">
+        <f>SUM(AA2:AA38)</f>
+        <v>8363344733890.2998</v>
+      </c>
+      <c r="AB39" s="13">
+        <f t="shared" si="1"/>
+        <v>5416674050.4470854</v>
       </c>
     </row>
   </sheetData>
@@ -8021,14 +8049,15 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4D5C567-F4F1-4D55-8262-44139A77B677}">
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="18.21875" bestFit="1" customWidth="1"/>
     <col min="4" max="10" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -8059,8 +8088,11 @@
       <c r="J1" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -8091,8 +8123,12 @@
       <c r="J2" s="11">
         <v>18498928176.209999</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2" s="13">
+        <f>SUM(D2,F2,H2,J2)</f>
+        <v>65813923395.540001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -8123,8 +8159,12 @@
       <c r="J3" s="11">
         <v>17011556718.549999</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3" s="13">
+        <f t="shared" ref="K3:K38" si="0">SUM(D3,F3,H3,J3)</f>
+        <v>63468914239.209991</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -8155,8 +8195,12 @@
       <c r="J4" s="11">
         <v>53584587922.209999</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4" s="13">
+        <f t="shared" si="0"/>
+        <v>172293623514.09</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -8187,8 +8231,12 @@
       <c r="J5" s="11">
         <v>19484900291.110001</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K5" s="13">
+        <f t="shared" si="0"/>
+        <v>71269337475.76001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -8219,8 +8267,12 @@
       <c r="J6" s="11">
         <v>15481399067.98</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K6" s="13">
+        <f t="shared" si="0"/>
+        <v>55360983478.830002</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -8251,8 +8303,12 @@
       <c r="J7" s="11">
         <v>52028452764.389999</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K7" s="13">
+        <f t="shared" si="0"/>
+        <v>173200463598.96002</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -8283,8 +8339,12 @@
       <c r="J8" s="11">
         <v>19372501657.73</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K8" s="13">
+        <f t="shared" si="0"/>
+        <v>68231268960.040009</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -8315,8 +8375,12 @@
       <c r="J9" s="11">
         <v>20027245563.349998</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K9" s="13">
+        <f t="shared" si="0"/>
+        <v>71133464608.200012</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -8347,8 +8411,12 @@
       <c r="J10" s="11">
         <v>12757875724.51</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K10" s="13">
+        <f t="shared" si="0"/>
+        <v>46721045613.080002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -8379,8 +8447,12 @@
       <c r="J11" s="11">
         <v>67807267304.610001</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K11" s="13">
+        <f t="shared" si="0"/>
+        <v>217841728279.88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -8411,8 +8483,12 @@
       <c r="J12" s="11">
         <v>14684667388.65</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K12" s="13">
+        <f t="shared" si="0"/>
+        <v>54819570748.040001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -8443,8 +8519,12 @@
       <c r="J13" s="11">
         <v>17343060816.610001</v>
       </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K13" s="13">
+        <f t="shared" si="0"/>
+        <v>63106598374.589996</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -8475,8 +8555,12 @@
       <c r="J14" s="11">
         <v>13983849026.85</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K14" s="13">
+        <f t="shared" si="0"/>
+        <v>49919252738.659996</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -8507,8 +8591,12 @@
       <c r="J15" s="11">
         <v>16421866385.27</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K15" s="13">
+        <f t="shared" si="0"/>
+        <v>59609631671.130005</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -8539,8 +8627,12 @@
       <c r="J16" s="11">
         <v>14330136812.33</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K16" s="13">
+        <f t="shared" si="0"/>
+        <v>51387410451.740005</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -8571,8 +8663,12 @@
       <c r="J17" s="11">
         <v>19681356196.790001</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K17" s="13">
+        <f t="shared" si="0"/>
+        <v>68640188884.040001</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -8603,8 +8699,12 @@
       <c r="J18" s="11">
         <v>18720348004.119999</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K18" s="13">
+        <f t="shared" si="0"/>
+        <v>72539598669.009995</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -8635,8 +8735,12 @@
       <c r="J19" s="11">
         <v>15902063503.530001</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K19" s="13">
+        <f t="shared" si="0"/>
+        <v>54649843790.360001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -8667,8 +8771,12 @@
       <c r="J20" s="11">
         <v>27313957678.040001</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K20" s="13">
+        <f t="shared" si="0"/>
+        <v>100139407045.64001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -8699,8 +8807,12 @@
       <c r="J21" s="11">
         <v>18970065788.619999</v>
       </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K21" s="13">
+        <f t="shared" si="0"/>
+        <v>68823435564.059998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -8731,8 +8843,12 @@
       <c r="J22" s="11">
         <v>17115244058.91</v>
       </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K22" s="13">
+        <f t="shared" si="0"/>
+        <v>64138354243.830002</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -8763,8 +8879,12 @@
       <c r="J23" s="11">
         <v>16733175590.85</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K23" s="13">
+        <f t="shared" si="0"/>
+        <v>62705013652.209999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -8795,8 +8915,12 @@
       <c r="J24" s="11">
         <v>15086296181.290001</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K24" s="13">
+        <f t="shared" si="0"/>
+        <v>56477916362.400002</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -8827,8 +8951,12 @@
       <c r="J25" s="11">
         <v>64709134590.809998</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K25" s="13">
+        <f t="shared" si="0"/>
+        <v>249601727263.69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -8859,8 +8987,12 @@
       <c r="J26" s="11">
         <v>15350379934.940001</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K26" s="13">
+        <f t="shared" si="0"/>
+        <v>58377192920.419998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -8891,8 +9023,12 @@
       <c r="J27" s="11">
         <v>17162172711.889999</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K27" s="13">
+        <f t="shared" si="0"/>
+        <v>63311366339.880005</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -8923,8 +9059,12 @@
       <c r="J28" s="11">
         <v>15326088992.75</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K28" s="13">
+        <f t="shared" si="0"/>
+        <v>52037706692.82</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -8955,8 +9095,12 @@
       <c r="J29" s="11">
         <v>20788171093.970001</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K29" s="13">
+        <f t="shared" si="0"/>
+        <v>73683078005.820007</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -8987,8 +9131,12 @@
       <c r="J30" s="11">
         <v>15207315375.209999</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K30" s="13">
+        <f t="shared" si="0"/>
+        <v>55266523105.260002</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -9019,8 +9167,12 @@
       <c r="J31" s="11">
         <v>26589558966.400002</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K31" s="13">
+        <f t="shared" si="0"/>
+        <v>95905559171.410004</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -9051,8 +9203,12 @@
       <c r="J32" s="11">
         <v>16117933023.200001</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K32" s="13">
+        <f t="shared" si="0"/>
+        <v>58668032487.860001</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -9083,8 +9239,12 @@
       <c r="J33" s="11">
         <v>55073733212.269997</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K33" s="13">
+        <f t="shared" si="0"/>
+        <v>190587569587.34998</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -9115,8 +9275,12 @@
       <c r="J34" s="11">
         <v>17616987565.73</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K34" s="13">
+        <f t="shared" si="0"/>
+        <v>63594841494.979996</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -9147,8 +9311,12 @@
       <c r="J35" s="11">
         <v>16165112078.57</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K35" s="13">
+        <f t="shared" si="0"/>
+        <v>58934482401.229996</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -9179,8 +9347,12 @@
       <c r="J36" s="11">
         <v>16502972733.9</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K36" s="13">
+        <f t="shared" si="0"/>
+        <v>59139521774.099998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -9211,8 +9383,12 @@
       <c r="J37" s="11">
         <v>17098727819.309999</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K37" s="13">
+        <f t="shared" si="0"/>
+        <v>62751617566.129997</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -9234,6 +9410,40 @@
       <c r="I38" s="11"/>
       <c r="J38" s="11">
         <v>24284532336.32</v>
+      </c>
+      <c r="K38" s="13">
+        <f t="shared" si="0"/>
+        <v>74674052915.559998</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="K39" s="13">
+        <f>SUM(K2:K38)</f>
+        <v>3048824247085.8096</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E14B4918-D611-41E8-B116-3595EBC3608C}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="10">
+        <f>SUM('2016'!AA39,'2017'!AA39,'2018'!AA39,'2019'!AA39,'2020'!AA39,'2021'!AA39,'2022'!AA39,'2023'!AA39,'2024'!AA39,'2025'!AA39,'2026'!K39)</f>
+        <v>37837640188697.211</v>
       </c>
     </row>
   </sheetData>
@@ -9243,14 +9453,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AD39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="26" width="18" customWidth="1"/>
     <col min="27" max="27" width="20.5546875" customWidth="1"/>
     <col min="28" max="28" width="21.109375" customWidth="1"/>
-    <col min="29" max="29" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="17.6640625" customWidth="1"/>
     <col min="30" max="30" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9528,7 +9738,7 @@
         <v>6201369567.2299995</v>
       </c>
       <c r="AC3" s="11">
-        <f t="shared" ref="AC3:AC38" si="1">AA3/305</f>
+        <f t="shared" ref="AC3:AC39" si="1">AA3/305</f>
         <v>128005606.88171281</v>
       </c>
       <c r="AD3" s="13">
@@ -12832,6 +13042,16 @@
       <c r="AD38" s="13">
         <f t="shared" si="2"/>
         <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AA39" s="10">
+        <f>SUM(AA2:AA38)</f>
+        <v>1881707854553.8848</v>
+      </c>
+      <c r="AC39" s="11">
+        <f t="shared" si="1"/>
+        <v>6169533949.3569994</v>
       </c>
     </row>
   </sheetData>
@@ -12841,14 +13061,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AD39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="26" width="18" customWidth="1"/>
     <col min="27" max="27" width="22.5546875" customWidth="1"/>
     <col min="28" max="28" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="17.44140625" customWidth="1"/>
     <col min="30" max="30" width="18" customWidth="1"/>
   </cols>
   <sheetData>
@@ -13120,7 +13340,7 @@
         <v>6204876665.6199999</v>
       </c>
       <c r="AC3" s="11">
-        <f t="shared" ref="AC3:AC38" si="1">AA3/306</f>
+        <f t="shared" ref="AC3:AC39" si="1">AA3/306</f>
         <v>161288777.44291016</v>
       </c>
       <c r="AD3" s="13">
@@ -16324,6 +16544,16 @@
       <c r="AD38" s="13">
         <f t="shared" si="2"/>
         <v>214116547.89156866</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AA39" s="10">
+        <f>SUM(AA2:AA38)</f>
+        <v>2565722147158.1523</v>
+      </c>
+      <c r="AC39" s="11">
+        <f t="shared" si="1"/>
+        <v>8384712899.2096481</v>
       </c>
     </row>
   </sheetData>
@@ -16333,7 +16563,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AD39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -16618,7 +16848,7 @@
         <v>9704650185.4200001</v>
       </c>
       <c r="AC3" s="11">
-        <f t="shared" ref="AC3:AC38" si="1">AA3/306</f>
+        <f t="shared" ref="AC3:AC39" si="1">AA3/306</f>
         <v>158731668.17641926</v>
       </c>
       <c r="AD3" s="13">
@@ -19925,6 +20155,16 @@
       <c r="AD38" s="13">
         <f t="shared" si="2"/>
         <v>243673793.57944444</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AA39" s="10">
+        <f>SUM(AA2:AA38)</f>
+        <v>2484908586961.2695</v>
+      </c>
+      <c r="AC39" s="11">
+        <f t="shared" si="1"/>
+        <v>8120616297.2590504</v>
       </c>
     </row>
   </sheetData>
@@ -19934,7 +20174,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AD39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -23528,6 +23768,12 @@
         <v>258594665.44219944</v>
       </c>
     </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AA39" s="10">
+        <f>SUM(AA2:AA38)</f>
+        <v>2267723055014.5493</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -23535,7 +23781,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AD39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -23820,11 +24066,11 @@
         <v>13011611228.120001</v>
       </c>
       <c r="AC3" s="10">
-        <f t="shared" ref="AC3:AC38" si="1">AA3/399</f>
+        <f t="shared" ref="AC3:AC39" si="1">AA3/399</f>
         <v>135671158.11363485</v>
       </c>
       <c r="AD3" s="11">
-        <f t="shared" ref="AD3:AD38" si="2">AA3/399</f>
+        <f t="shared" ref="AD3:AD39" si="2">AA3/399</f>
         <v>135671158.11363485</v>
       </c>
     </row>
@@ -27126,6 +27372,20 @@
       <c r="AD38" s="11">
         <f t="shared" si="2"/>
         <v>161897139.10460377</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AA39" s="10">
+        <f>SUM(AA2:AA38)</f>
+        <v>2517703969009.021</v>
+      </c>
+      <c r="AC39" s="10">
+        <f t="shared" si="1"/>
+        <v>6310035010.0476713</v>
+      </c>
+      <c r="AD39" s="11">
+        <f t="shared" si="2"/>
+        <v>6310035010.0476713</v>
       </c>
     </row>
   </sheetData>
@@ -27135,7 +27395,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A16A8713-F30F-4E2A-A603-CBB41D121E4D}">
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AD39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="26" width="17.21875" bestFit="1" customWidth="1"/>
@@ -27419,7 +27679,7 @@
         <v>13175774969.529999</v>
       </c>
       <c r="AC3" s="13">
-        <f t="shared" ref="AC3:AC38" si="1">AA3/423</f>
+        <f t="shared" ref="AC3:AC39" si="1">AA3/423</f>
         <v>142295386.54900709</v>
       </c>
       <c r="AD3" s="13">
@@ -30732,6 +30992,16 @@
       <c r="AD38" s="13">
         <f t="shared" si="2"/>
         <v>294011287.27955085</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AA39" s="13">
+        <f>SUM(AA2:AA38)</f>
+        <v>3403240943317.7603</v>
+      </c>
+      <c r="AC39" s="13">
+        <f t="shared" si="1"/>
+        <v>8045486863.6353674</v>
       </c>
     </row>
   </sheetData>
@@ -30741,7 +31011,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F72DB5A-21C0-4DBA-BADB-D83EE6FFFFD8}">
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AD39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="26" width="17.21875" bestFit="1" customWidth="1"/>
@@ -31025,7 +31295,7 @@
         <v>17066189975.839998</v>
       </c>
       <c r="AC3" s="13">
-        <f t="shared" ref="AC3:AC38" si="1">AA3/646</f>
+        <f t="shared" ref="AC3:AC39" si="1">AA3/646</f>
         <v>120664820.27356037</v>
       </c>
       <c r="AD3" s="13">
@@ -34330,6 +34600,16 @@
       <c r="AD38" s="13">
         <f t="shared" si="2"/>
         <v>326780631.79003096</v>
+      </c>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AA39" s="13">
+        <f>SUM(AA2:AA38)</f>
+        <v>4005256605143.8892</v>
+      </c>
+      <c r="AC39" s="13">
+        <f t="shared" si="1"/>
+        <v>6200087624.0617476</v>
       </c>
     </row>
   </sheetData>
@@ -34339,12 +34619,11 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C348C43-16CC-4A1A-AD98-6F32B18E9372}">
-  <dimension ref="A1:AD38"/>
+  <dimension ref="A1:AD39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="26" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="18.21875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="18.109375" customWidth="1"/>
     <col min="30" max="30" width="16.88671875" customWidth="1"/>
   </cols>
@@ -34623,7 +34902,7 @@
         <v>20298222818.559998</v>
       </c>
       <c r="AC3" s="13">
-        <f t="shared" ref="AC3:AC38" si="1">AA3/1480</f>
+        <f t="shared" ref="AC3:AC39" si="1">AA3/1480</f>
         <v>76158330.659844592</v>
       </c>
       <c r="AD3" s="13">
@@ -37931,6 +38210,16 @@
         <v>190786523.66604054</v>
       </c>
     </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.3">
+      <c r="AA39" s="13">
+        <f>SUM(AA2:AA38)</f>
+        <v>5949233422223.8584</v>
+      </c>
+      <c r="AC39" s="13">
+        <f t="shared" si="1"/>
+        <v>4019752312.3134179</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>